<commit_message>
fix: 3.1 thêm NTID vào điều chuyển
</commit_message>
<xml_diff>
--- a/static/uploads/mau/dieuchuyen/dieuchuyen.xlsx
+++ b/static/uploads/mau/dieuchuyen/dieuchuyen.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Phanmem\HRM\static\uploads\mau\dieuchuyen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\HRM\static\uploads\mau\dieuchuyen\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA0F918-735C-494A-936D-CC383A46F376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,21 +21,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Mã số thẻ</t>
   </si>
@@ -73,12 +65,15 @@
   </si>
   <si>
     <t>Rút hồ sơ</t>
+  </si>
+  <si>
+    <t>NTID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -463,19 +458,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -494,8 +489,11 @@
       <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>13295</v>
       </c>
@@ -511,8 +509,11 @@
       <c r="E2" s="2">
         <v>45516</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>12543</v>
       </c>
@@ -528,10 +529,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
@@ -544,29 +546,29 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>

</xml_diff>